<commit_message>
data: update 2026-09-17 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/daily_logs/daily_2026-09-17.xlsx
+++ b/daily_logs/daily_2026-09-17.xlsx
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F12" s="24" t="n">
         <v>23</v>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.62</v>
+        <v>2.68</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>-18</v>
+        <v>-27</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>5</v>
+        <v>5.01</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-28</v>
+        <v>-30</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.36</v>
+        <v>5.35</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.31</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>-26</v>
+        <v>-28</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1716,7 +1716,7 @@
         </is>
       </c>
       <c r="E41" s="24" t="n">
-        <v>3.5</v>
+        <v>3.75</v>
       </c>
       <c r="F41" s="24" t="n"/>
       <c r="G41" s="6" t="n"/>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.64</v>
+        <v>3.62</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -1886,10 +1886,10 @@
         </is>
       </c>
       <c r="E47" s="24" t="n">
-        <v>2991.31</v>
+        <v>3013.79</v>
       </c>
       <c r="F47" s="24" t="n">
-        <v>-89.48</v>
+        <v>-95.19</v>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
@@ -1981,10 +1981,10 @@
         </is>
       </c>
       <c r="E50" s="24" t="n">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F50" s="24" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G50" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>-1</v>
+        <v>3</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2471,10 +2471,10 @@
         </is>
       </c>
       <c r="E66" s="24" t="n">
-        <v>6.76</v>
+        <v>6.95</v>
       </c>
       <c r="F66" s="24" t="n">
-        <v>-53</v>
+        <v>-65</v>
       </c>
       <c r="G66" s="6" t="n"/>
     </row>
@@ -2914,12 +2914,12 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=-1.0bp [OK]
-HY OAS 5dd=-9.0bp
-HYG 5d=nan% [OK]
+          <t>HY OAS 20dd=3.0bp [OK]
+HY OAS 5dd=1.0bp
+HYG 5d=-0.7% [OK]
 HYG DD%=None% max drawdown
-FXY 5d=nan% [OK]
-SPY vs 200MA: above ($SPY=nan, 200MA=nan)
+FXY 5d=-1.6% [OK]
+SPY vs 200MA: above ($SPY=754.0499877929688, 200MA=713.4)
 Extreme: VIX&gt;35•HYOAS&gt;5%•SOFR-IORB&gt;+5bp</t>
         </is>
       </c>

</xml_diff>